<commit_message>
added hw05-access, updated tutorial excel file
</commit_message>
<xml_diff>
--- a/LEC/lec10-access-tutorial/employee.xlsx
+++ b/LEC/lec10-access-tutorial/employee.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25427"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\EDU-VFP-E-001\Users\IFrommer\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgacademy-my.sharepoint.com/personal/ian_frommer_uscga_edu/Documents/Documents/github/info_sys_course/LEC/lec10-access-tutorial/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0969DE7F-0862-4C1B-B510-48D46AFAC375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{0969DE7F-0862-4C1B-B510-48D46AFAC375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11C7A896-7C1B-4F71-9B41-90EFE8C32E0B}"/>
   <bookViews>
-    <workbookView xWindow="29880" yWindow="2670" windowWidth="18000" windowHeight="9240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2685" yWindow="2280" windowWidth="26235" windowHeight="13185" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Employee" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="44">
   <si>
     <t>Last Name</t>
   </si>
@@ -64,24 +64,6 @@
     <t>19702</t>
   </si>
   <si>
-    <t>CT</t>
-  </si>
-  <si>
-    <t>06320</t>
-  </si>
-  <si>
-    <t>Smith</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>12340</t>
-  </si>
-  <si>
-    <t>22 Maple Dr</t>
-  </si>
-  <si>
     <t>Baltimore</t>
   </si>
   <si>
@@ -160,16 +142,16 @@
     <t>Santiago</t>
   </si>
   <si>
-    <t>Urlastname</t>
-  </si>
-  <si>
-    <t>Urfirstname</t>
-  </si>
-  <si>
-    <t>27 Mohegan Ave</t>
-  </si>
-  <si>
-    <t>New London</t>
+    <t>Stu</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>1 Pequot Ave</t>
+  </si>
+  <si>
+    <t>Elkton</t>
   </si>
 </sst>
 </file>
@@ -386,9 +368,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -426,9 +408,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -461,26 +443,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -513,26 +478,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -706,18 +654,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="15.54296875" customWidth="1"/>
-    <col min="3" max="3" width="14.08984375" customWidth="1"/>
-    <col min="4" max="4" width="21.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="14.08984375" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -746,12 +694,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
@@ -769,180 +717,154 @@
         <v>13</v>
       </c>
       <c r="H2" s="3">
-        <v>42156</v>
+        <v>43252</v>
       </c>
       <c r="I2" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:9" ht="21" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="3">
+        <v>36312</v>
+      </c>
+      <c r="I3" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="21" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="I3" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H4" s="3">
-        <v>36312</v>
+        <v>32704</v>
       </c>
       <c r="I4" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H5" s="3">
-        <v>32704</v>
+        <v>40009</v>
       </c>
       <c r="I5" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="21" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="H6" s="3">
-        <v>40009</v>
+        <v>42962</v>
       </c>
       <c r="I6" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>22</v>
+    <row r="7" spans="1:9" s="8" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="8">
+        <v>21921</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="9">
+        <v>21921</v>
       </c>
       <c r="H7" s="3">
-        <v>42962</v>
-      </c>
-      <c r="I7" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" s="8" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="8">
-        <v>9911</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="3">
         <v>38579</v>
       </c>
-      <c r="I8" s="7" t="b">
+      <c r="I7" s="7" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>